<commit_message>
Populate spreadsheet with state DOE financial literacy contacts
Added contact information for 24 states from web research:

Tier 1 (Imminent Mandates):
- California: CDE Personal Finance division
- Ohio: Jessee Hankins, FL-Social Studies Specialist
- Pennsylvania: Bureau of Curriculum
- Wisconsin: Jennifer Jackson, Education Consultant

Tier 2 (Strong Relationships):
- Oklahoma: Brenda Beymer-Chapman, Project Manager
- Texas: TEKS Curriculum division
- Florida: Pedro Hernandez, OSFA
- Colorado: Stephanie Hartman, FL Specialist

Tier 3 (Established): Added contacts for AR, GA, KY, NC, NJ, SC,
TN, UT, VA and others with available FL resources page URLs

Data gathered from official state DOE websites and web searches.

https://claude.ai/code/session_01PvVz8P6ksgRvV14Gy7UGhf
</commit_message>
<xml_diff>
--- a/State_DOE_Backlink_Outreach_Tracker.xlsx
+++ b/State_DOE_Backlink_Outreach_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1 - Imminent" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 2 - Relationships" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 3 - Established" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email Template" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tier 1 - Imminent" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tier 2 - Relationships" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tier 3 - Established" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Email Template" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,11 +535,31 @@
           <t>cde.ca.gov</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Curriculum Frameworks Division</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Personal Finance Curriculum</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>916-319-0881</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>PersonalFinance@cde.ca.gov</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cde.ca.gov/ci/cr/cf/personalfinance.asp</t>
+        </is>
+      </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -563,11 +583,27 @@
           <t>education.ohio.gov</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Jessee Hankins</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Financial Literacy-Social Studies Specialist</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Financial.Literacy@education.ohio.gov</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://education.ohio.gov/Topics/Learning-in-Ohio/Financial-Literacy</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -591,11 +627,27 @@
           <t>pa.gov/education</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Bureau of Curriculum</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Curriculum, Assessment and Instruction</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>717-783-2193</t>
+        </is>
+      </c>
       <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pdesas.org/Page/Viewer/ViewPage/81/</t>
+        </is>
+      </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -619,11 +671,31 @@
           <t>dpi.wi.gov</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Jennifer Jackson</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Education Consultant, Business &amp; IT</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>608-266-2803</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>jennifer.jackson@dpi.wi.gov</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://dpi.wi.gov/bit</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -735,11 +807,31 @@
           <t>sde.ok.gov</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Brenda Beymer-Chapman, J.D.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Project Manager, Social Studies &amp; PFL</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>405-522-3523</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Brenda.Chapman@sde.ok.gov</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://oklahoma.gov/education/services/standards-learning/personal-financial-literacy.html</t>
+        </is>
+      </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -763,11 +855,31 @@
           <t>tea.texas.gov</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Curriculum Standards Division</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>TEKS Curriculum</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>512-463-9581</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>teks@tea.texas.gov</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://tea.texas.gov/academics/subject-areas/social-studies/</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -791,11 +903,31 @@
           <t>fldoe.org</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Pedro Hernandez</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Office of Student Financial Assistance</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>850-410-5200</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Pedro.Hernandez@fldoe.org</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fldoe.org/</t>
+        </is>
+      </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -819,11 +951,27 @@
           <t>cde.state.co.us</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Stephanie Hartman</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Financial Literacy Specialist</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>720-739-3238</t>
+        </is>
+      </c>
       <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cde.state.co.us/cofinancialliteracy</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -935,11 +1083,23 @@
           <t>alsde.edu</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ALSDE Career Preparedness</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Career and Technical Education</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.alabamaachieves.org/</t>
+        </is>
+      </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -963,11 +1123,31 @@
           <t>dese.ade.arkansas.gov</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Amber Murry Pirnique, M.Ed.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Disciplinary Literacy Program Manager</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>501-682-5764</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Amber.Pirnique@ade.arkansas.gov</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://dese.ade.arkansas.gov/Offices/learning-services/curriculum-support/personal-finance</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -995,7 +1175,11 @@
       <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>https://portal.ct.gov/sde</t>
+        </is>
+      </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1023,7 +1207,11 @@
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.doe.k12.de.us/</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1047,11 +1235,27 @@
           <t>gadoe.org</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Social Studies Team</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>GaDOE Social Studies</t>
+        </is>
+      </c>
       <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>socialstudies@doe.k12.ga.us</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>https://gadoe.org/learning/social-studies/</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1079,7 +1283,11 @@
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sde.idaho.gov/</t>
+        </is>
+      </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1103,11 +1311,27 @@
           <t>isbe.net</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>ISBE Curriculum Division</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Consumer Education</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>217-557-4723</t>
+        </is>
+      </c>
       <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.isbe.net/</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1131,11 +1355,23 @@
           <t>in.gov/doe</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Eric Ogle / Peggy Wild</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Financial Literacy Education</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.in.gov/doe/students/indiana-academic-standards/financial-literacy/</t>
+        </is>
+      </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1163,7 +1399,11 @@
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>https://educateiowa.gov/</t>
+        </is>
+      </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1187,11 +1427,31 @@
           <t>education.ky.gov</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Heather Ransom</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Academic Program Consultant, Social Studies</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>502-564-2106 x4130</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>heather.ransom@education.ky.gov</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.education.ky.gov/curriculum/conpro/Pages/FinLit.aspx</t>
+        </is>
+      </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1215,11 +1475,27 @@
           <t>louisianabelieves.com</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>LDOE Teaching &amp; Learning</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Financial Literacy</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>877-453-2721</t>
+        </is>
+      </c>
       <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>https://doe.louisiana.gov/</t>
+        </is>
+      </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1243,11 +1519,27 @@
           <t>michigan.gov/mde</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>MDE Personal Finance</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Academic Standards</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>517-241-5000</t>
+        </is>
+      </c>
       <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.michigan.gov/mde/services/academic-standards/personal-finance</t>
+        </is>
+      </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1327,11 +1619,27 @@
           <t>dese.mo.gov</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr"/>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>DESE BMIT</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Personal Finance Curriculum</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>573-751-4234</t>
+        </is>
+      </c>
       <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>https://dese.mo.gov/bmit-personal-finance</t>
+        </is>
+      </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1383,11 +1691,23 @@
           <t>education.ne.gov</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr"/>
-      <c r="D20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>NDE Social Studies</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Financial Literacy Act</t>
+        </is>
+      </c>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3" t="inlineStr"/>
-      <c r="G20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.education.ne.gov/socialstudies/financial-literacy-act-guidance/</t>
+        </is>
+      </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1439,11 +1759,27 @@
           <t>nj.gov/education</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr"/>
-      <c r="D22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Office of Career Readiness</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Career Readiness</t>
+        </is>
+      </c>
       <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>CTE@doe.nj.gov</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nj.gov/education/standards/clicks/finlit.shtml</t>
+        </is>
+      </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1495,11 +1831,23 @@
           <t>dpi.nc.gov</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr"/>
-      <c r="D24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Lori Major Carlin</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Section Chief, Social Studies &amp; Arts Ed</t>
+        </is>
+      </c>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="3" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr"/>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.dpi.nc.gov/</t>
+        </is>
+      </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1579,11 +1927,31 @@
           <t>ed.sc.gov</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
-      <c r="G27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Reece Spradley</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Social Studies Education Associate</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>803-734-8335</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>rcspradley@ed.sc.gov</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>https://ed.sc.gov/instruction/standards/social-studies/financial-literacy/</t>
+        </is>
+      </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1607,11 +1975,23 @@
           <t>tn.gov/education</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr"/>
-      <c r="D28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>TN Financial Literacy Commission</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Department of Treasury</t>
+        </is>
+      </c>
       <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="3" t="inlineStr"/>
-      <c r="G28" s="3" t="inlineStr"/>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>https://treasury.tn.gov/Financial-Education</t>
+        </is>
+      </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1635,11 +2015,31 @@
           <t>schools.utah.gov</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>April Painter</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Education Specialist, General Financial Literacy</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>801-538-7750</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>April.Painter@schools.utah.gov</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>https://schools.utah.gov/cte/gfl</t>
+        </is>
+      </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
           <t>🔴</t>
@@ -1663,11 +2063,31 @@
           <t>doe.virginia.gov</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr"/>
-      <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr"/>
-      <c r="G30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Judith Sams</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Specialist, Business &amp; IT</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>804-371-0196</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Judith.Sams@doe.virginia.gov</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.doe.virginia.gov/teaching-learning-assessment/instruction/economics-personal-finance</t>
+        </is>
+      </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
           <t>🔴</t>

</xml_diff>

<commit_message>
Add Texas ESC Regions sheet with all 20 regional contacts
Added new sheet with all 20 Texas Education Service Centers:
- Region 1 (Edinburg) through Region 20 (San Antonio)
- Includes Executive Director names, addresses, phone/fax
- Status column for tracking outreach

Key regions for PFL Academy:
- Region 4: Houston (Dr. Rodney Watson)
- Region 10: Dallas/Richardson (Dr. Jana Melsheimer)
- Region 11: Fort Worth (Dr. Clyde Steelman Jr.)
- Region 13: Austin (Dr. Rich Elsasser)
- Region 20: San Antonio (Dr. Claudia Gonzalez)

https://claude.ai/code/session_01PvVz8P6ksgRvV14Gy7UGhf
</commit_message>
<xml_diff>
--- a/State_DOE_Backlink_Outreach_Tracker.xlsx
+++ b/State_DOE_Backlink_Outreach_Tracker.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Tier 2 - Relationships" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Tier 3 - Established" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Email Template" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Texas ESC Regions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2263,4 +2264,806 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>City/Area</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Fax</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Region 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Edinburg</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dr. Daniel King</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1900 West Schunior, Edinburg, TX 78541</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>(956) 984-6001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>(956) 984-7655</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Region 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Corpus Christi</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Dr. Esperanza Zendejas</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>209 North Water Street, Corpus Christi, TX 78401</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>(361) 561-8400</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>(361) 883-3442</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Region 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Victoria</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Dr. Morris Lyons</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1905 Leary Lane, Victoria, TX 77901</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>(361) 573-0731</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>(361) 576-4804</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Region 4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Dr. Rodney Watson</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>7145 West Tidwell, Houston, TX 77092</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>(713) 462-7708</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>(713) 744-6514</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Region 5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Beaumont</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Dr. Byron Terrier</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>350 Pine Street, Suite 500, Beaumont, TX 77701</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>(409) 951-1700</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>(409) 951-1800</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Region 6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Huntsville</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mr. Michael Holland</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3332 Montgomery Road, Huntsville, TX 77340</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>(936) 435-8400</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>(936) 435-8484</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Region 7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kilgore</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mr. Todd Schneider</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1909 N. Longview Street, Kilgore, TX 75662</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>(903) 988-6700</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>(903) 988-6708</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Region 8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pittsburg</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Dr. David W. Fitts</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>4845 U.S. Highway 271 N., Pittsburg, TX 75686</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>(903) 572-8551</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>(903) 575-2611</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Region 9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wichita Falls</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mr. West Pierce</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>301 Loop 11, Wichita Falls, TX 76306</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>(940) 322-6928</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>(940) 767-3836</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Region 10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Richardson/Dallas</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Dr. Jana Melsheimer</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>400 E. Spring Valley Road, Richardson, TX 75081</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>(972) 348-1700</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>(972) 231-3642</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Region 11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Dr. Clyde Steelman, Jr.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1451 S. Cherry Lane, White Settlement, TX 76108</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>(817) 740-3600</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>(817) 740-7600</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Region 12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Waco</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mr. Kenny Berry</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2101 W. Loop 340, Waco, TX 76712</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>(254) 297-1212</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>(254) 666-0823</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Region 13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dr. Rich Elsasser</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>5701 Springdale Road, Austin, TX 78723</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>(512) 919-5313</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>(512) 919-5374</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Region 14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Abilene</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mr. Chris Wigington</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1850 Highway 351, Abilene, TX 79601</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>(325) 675-8600</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>(325) 675-8659</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Region 15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>San Angelo</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Dr. Casey Callahan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>612 South Irene Street, San Angelo, TX 76903</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>(325) 658-6571</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>(325) 655-4823</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Region 16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Amarillo</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Dr. Tanya Larkin</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>5800 Bell Street, Amarillo, TX 79109</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>(806) 677-5000</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>(806) 677-5001</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Region 17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lubbock</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Mr. Kyle Wargo</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1111 West Loop 289, Lubbock, TX 79416</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>(806) 792-4000</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>(806) 792-1523</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Region 18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Midland</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Dr. Dewitt Smith</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2811 LaForce Blvd., Midland, TX 79706</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>(432) 563-2380</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>(432) 567-3290</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Region 19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>El Paso</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Dr. Armando Aguirre</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>6611 Boeing Drive, El Paso, TX 79925</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>(915) 780-1919</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>(915) 780-6537</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Region 20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Dr. Claudia Gonzalez</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>1314 Hines Ave, San Antonio, TX 78208</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>(210) 370-5200</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>